<commit_message>
Tarnoc v2: base ramp slowed to ~310 / 1,100 / 3,300 / 7,200 units via the marketing table; summary text updated
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-07.xlsx
+++ b/models/Tarnoc_v2_2026-09-07.xlsx
@@ -1155,7 +1155,7 @@
     <row r="35">
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Base, EUR3m: 7,400 units and EUR126m revenue in 2030, EBITDA negative until 2030 (EUR18m), 87 people, cash low of -EUR0.25m in December 2029.</t>
+          <t>Base, EUR3m: 310 units in 2027, 1,100 in 2028, 3,300 in 2029, 7,200 in 2030 (EUR123m revenue). EBITDA negative until 2030 (EUR18m), 84 people, cash low of -EUR1.4m in December 2029.</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
     <row r="50">
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Base on EUR3m runs out of cash at the end of 2029. It needs a bigger raise, the two-year BOM pricing, or the extra marketing push above.</t>
+          <t>Base on EUR3m runs out of cash during 2028 and is EUR1.4m short at the end of 2029. It needs a raise of about EUR5m, or the two-year BOM pricing.</t>
         </is>
       </c>
     </row>
@@ -3744,16 +3744,16 @@
         <v>0</v>
       </c>
       <c r="E48" s="32" t="n">
-        <v>28000</v>
+        <v>13000</v>
       </c>
       <c r="F48" s="32" t="n">
-        <v>70000</v>
+        <v>35000</v>
       </c>
       <c r="G48" s="32" t="n">
-        <v>120000</v>
+        <v>85000</v>
       </c>
       <c r="H48" s="32" t="n">
-        <v>170000</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
Tarnoc v2: base deploys more of the raise: R&D 4/3 in 2027-28, partners 1/month and reps 0.5/month in 2027, field engineers 1 per 600 units; summary updated
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-07.xlsx
+++ b/models/Tarnoc_v2_2026-09-07.xlsx
@@ -4929,7 +4929,7 @@
         <v>0</v>
       </c>
       <c r="E60" s="47" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="F60" s="47" t="n">
         <v>0.25</v>
@@ -5033,7 +5033,7 @@
         <v>0</v>
       </c>
       <c r="E64" s="49" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F64" s="49" t="n">
         <v>1.5</v>
@@ -5855,10 +5855,10 @@
         <v>0</v>
       </c>
       <c r="E99" s="41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F99" s="41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G99" s="41" t="n">
         <v>3</v>
@@ -6165,10 +6165,10 @@
         </is>
       </c>
       <c r="D112" s="41" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="E112" s="41" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="F112" s="42">
         <f>IF(Assumptions!$E$5=2,E112,D112)</f>
@@ -6176,7 +6176,7 @@
       </c>
       <c r="J112" s="30" t="inlineStr">
         <is>
-          <t>sizes the field service team: units on a service contract divided by this number = engineers to hire. Each unit gets one visit a year, an engineer does three to four a day</t>
+          <t>sizes the field service team: units on a service contract divided by this number = engineers to hire. Each unit gets one visit a year plus breakdown cover; market range 600 to 900</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tarnoc v2: summary text and doc updated for the base package
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-07.xlsx
+++ b/models/Tarnoc_v2_2026-09-07.xlsx
@@ -1205,21 +1205,21 @@
     <row r="38">
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Base, EUR3m: 310 / 1,200 / 3,900 / 7,200 units in 2027 to 2030, EUR123m revenue in 2030. Gross margin 10%, 25%, 37%, 37%. EBITDA -2.1m, +1.0m, +17m, +34m. 85 people.</t>
+          <t>Base, EUR3m: 350 / 1,350 / 4,100 / 7,400 units in 2027 to 2030, EUR127m revenue in 2030. Gross margin 10%, 25%, 37%, 37%. EBITDA -2.5m, +0.8m, +18m, +34m. 95 people.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Cash low EUR0.9m in December 2027, about four months of cost; 69% of the raise used.</t>
+          <t xml:space="preserve">     Cash low EUR0.6m in December 2027, about two months of cost; 81% of the raise used.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Aggressive, EUR10m: 2,800 / 6,900 / 11,700 / 18,800 units, EUR321m revenue in 2030. Gross margin 28%, 38%, 37%, 37%. EBITDA +4.8m, +23m, +45m, +80m. 289 people.</t>
+          <t>Aggressive, EUR10m: 2,800 / 6,900 / 11,700 / 18,800 units, EUR321m revenue in 2030. Gross margin 28%, 38%, 37%, 37%. EBITDA +4.8m, +23m, +45m, +79m. 301 people.</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
     <row r="47">
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Soft spot 1. Base turns on about 100 units: 2028 plus 2029 volume is 5,100 against a 5,000 tier. At 4,900, 2028 costs EUR2,900 more per unit and EBITDA goes back to about -2.7m.</t>
+          <t>Soft spot 1. Base turns on about 500 units: 2028 plus 2029 volume is 5,500 against a 5,000 tier. Below 5,000, 2028 costs EUR2,900 more per unit and EBITDA goes back to about -3m.</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
     <row r="90">
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>Base: the 5,000-unit cliff in 2028. A one-quarter delay in the 2029 ramp is enough to miss it, and with it the year's margin step.</t>
+          <t>Base: the 5,000-unit cliff in 2028 (2028 plus 2029 volume is 5,500 against the 5,000 tier) and two months of cash cover in December 2027. A one-quarter delay in the 2029 ramp costs the margin step.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tarnoc v2: build-capacity block marked aggressive-only; marketer ratio relabelled and set to EUR1.5m per head
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-07.xlsx
+++ b/models/Tarnoc_v2_2026-09-07.xlsx
@@ -5371,7 +5371,7 @@
     <row r="78">
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>BUILD CAPACITY AND CAPEX  (assembly partner first, in-house takes over)</t>
+          <t>BUILD CAPACITY AND CAPEX  (assembly partner in both cases; in-house lines and capex in the aggressive case only)</t>
         </is>
       </c>
       <c r="C78" s="2" t="n"/>
@@ -5508,6 +5508,11 @@
         <f>IF(Assumptions!$E$5=2,E83,D83)</f>
         <v/>
       </c>
+      <c r="J83" s="30" t="inlineStr">
+        <is>
+          <t>aggressive only: the base case has no in-house line, so rows 83 to 89 do nothing in base</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="6" t="inlineStr">
@@ -5532,7 +5537,7 @@
       </c>
       <c r="J84" s="30" t="inlineStr">
         <is>
-          <t>EUR250 per unit of annual capacity; peers run EUR250 to 600</t>
+          <t>aggressive only. EUR250 per unit of annual capacity; peers run EUR250 to 600</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5564,7 @@
       </c>
       <c r="J85" s="30" t="inlineStr">
         <is>
-          <t>automated test, balancing and handling, which is why a line runs on 25 operators rather than 35</t>
+          <t>aggressive only. Automated test, balancing and handling, which is why a line runs on 25 operators rather than 35</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5645,7 @@
       </c>
       <c r="J88" s="30" t="inlineStr">
         <is>
-          <t>the building and the machines, not the people</t>
+          <t>aggressive only: the building and the machines, not the people</t>
         </is>
       </c>
     </row>
@@ -5664,6 +5669,11 @@
       <c r="F89" s="42">
         <f>IF(Assumptions!$E$5=2,E89,D89)</f>
         <v/>
+      </c>
+      <c r="J89" s="30" t="inlineStr">
+        <is>
+          <t>aggressive only: the base case has no fixed assets</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -6111,7 +6121,7 @@
     <row r="110">
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Marketing spend per marketer</t>
+          <t>Yearly marketing budget one marketer can run</t>
         </is>
       </c>
       <c r="C110" s="28" t="inlineStr">
@@ -6120,14 +6130,19 @@
         </is>
       </c>
       <c r="D110" s="33" t="n">
-        <v>3000000</v>
+        <v>1500000</v>
       </c>
       <c r="E110" s="33" t="n">
-        <v>3000000</v>
+        <v>1500000</v>
       </c>
       <c r="F110" s="34">
         <f>IF(Assumptions!$E$5=2,E110,D110)</f>
         <v/>
+      </c>
+      <c r="J110" s="30" t="inlineStr">
+        <is>
+          <t>sizes the marketing team only: the floor above plus one more person for every EUR1.5m of yearly spend. Not a spend. Benchmarks: one marketer per EUR1-1.5m of media</t>
+        </is>
       </c>
     </row>
     <row r="111">

</xml_diff>

<commit_message>
Tarnoc v2: fork into base-only and aggressive-only workbooks (MODE=base|aggr); single Value column, no switch, base has no in-house block anywhere; audit scripts handle both shapes
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-07.xlsx
+++ b/models/Tarnoc_v2_2026-09-07.xlsx
@@ -1548,12 +1548,12 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>2 + 1 per EUR3m spend</t>
+          <t>2 + 1 per EUR1.5m of yearly spend</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>supported</t>
         </is>
       </c>
       <c r="E63" s="17" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="E84" s="17" t="inlineStr">
         <is>
-          <t>For 289 staff, 14-22; HR alone needs 4-6</t>
+          <t>Fine for 95 staff; for 300 staff 14-22, and HR alone needs 4-6</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="J83" s="30" t="inlineStr">
         <is>
-          <t>aggressive only: the base case has no in-house line, so rows 83 to 89 do nothing in base</t>
+          <t>aggressive only: the base case has no in-house line, so the rows below do nothing in base</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tarnoc v2: reps and installer partners are whole people
Revenue Forecast rows 16 and 19 carried the planned rate (0.5 reps a month in
base 2027, 1.5 partners a month in base 2028) and rows 17 and 20 accumulated it,
so the model showed half a rep and half a partner. Base had a fractional
headcount in 33 of 60 months, aggressive in 15.

Rows 16 and 19 are now labelled as rates; rows 17 and 20 floor the running total,
so half a rep a month is one rep every second month. Shadow model updated to
match. All three workbooks rebuilt, full four-phase audit passed on each.

Base moves slightly: 2028 units 1,350 to 1,344, 2030 units 7,418 to 7,407, cash
low EUR571k to EUR599k, raise used 81% to 80%. Aggressive volumes unchanged.

Docs updated, plus a client-facing summary and an engagement summary.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M1MCemVM7wdLSxoFdkoz1t
</commit_message>
<xml_diff>
--- a/models/Tarnoc_v2_2026-09-07.xlsx
+++ b/models/Tarnoc_v2_2026-09-07.xlsx
@@ -1205,21 +1205,21 @@
     <row r="38">
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Base, EUR3m: 350 / 1,350 / 4,100 / 7,400 units in 2027 to 2030, EUR127m revenue in 2030. Gross margin 10%, 25%, 37%, 37%. EBITDA -2.5m, +0.8m, +18m, +34m. 95 people.</t>
+          <t>Base, EUR3m: 354 / 1,344 / 4,122 / 7,407 units in 2027 to 2030, EUR126m revenue in 2030. Gross margin 10%, 25%, 37%, 37%. EBITDA -2.5m, +0.9m, +17m, +34m. 95 people.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Cash low EUR0.6m in December 2027, about two months of cost; 81% of the raise used.</t>
+          <t xml:space="preserve">     Cash low EUR0.6m in December 2027, about two months of cost; 80% of the raise used.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Aggressive, EUR10m: 2,800 / 6,900 / 11,700 / 18,800 units, EUR321m revenue in 2030. Gross margin 28%, 38%, 37%, 37%. EBITDA +4.8m, +23m, +45m, +79m. 301 people.</t>
+          <t>Aggressive, EUR10m: 2,812 / 6,864 / 11,730 / 18,780 units, EUR321m revenue in 2030. Gross margin 28%, 38%, 37%, 37%. EBITDA +4.8m, +23m, +45m, +79m. 302 people.</t>
         </is>
       </c>
     </row>
@@ -23655,12 +23655,12 @@
     <row r="16">
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Reps hired</t>
+          <t>Rep hiring rate</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>FTE</t>
+          <t>FTE/month</t>
         </is>
       </c>
       <c r="E16" s="66">
@@ -23925,7 +23925,7 @@
       </c>
       <c r="BT16" s="30" t="inlineStr">
         <is>
-          <t>no sales reps before the first month we can sell</t>
+          <t>the planned rate, which can be less than one a month</t>
         </is>
       </c>
     </row>
@@ -23941,243 +23941,243 @@
         </is>
       </c>
       <c r="E17" s="13">
-        <f>Assumptions!$F$72+E16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:E16),0)</f>
         <v/>
       </c>
       <c r="F17" s="13">
-        <f>E17+F16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:F16),0)</f>
         <v/>
       </c>
       <c r="G17" s="13">
-        <f>F17+G16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:G16),0)</f>
         <v/>
       </c>
       <c r="H17" s="13">
-        <f>G17+H16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:H16),0)</f>
         <v/>
       </c>
       <c r="I17" s="13">
-        <f>H17+I16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:I16),0)</f>
         <v/>
       </c>
       <c r="J17" s="13">
-        <f>I17+J16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:J16),0)</f>
         <v/>
       </c>
       <c r="K17" s="13">
-        <f>J17+K16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:K16),0)</f>
         <v/>
       </c>
       <c r="L17" s="13">
-        <f>K17+L16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:L16),0)</f>
         <v/>
       </c>
       <c r="M17" s="13">
-        <f>L17+M16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:M16),0)</f>
         <v/>
       </c>
       <c r="N17" s="13">
-        <f>M17+N16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:N16),0)</f>
         <v/>
       </c>
       <c r="O17" s="13">
-        <f>N17+O16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:O16),0)</f>
         <v/>
       </c>
       <c r="P17" s="13">
-        <f>O17+P16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:P16),0)</f>
         <v/>
       </c>
       <c r="Q17" s="13">
-        <f>P17+Q16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:Q16),0)</f>
         <v/>
       </c>
       <c r="R17" s="13">
-        <f>Q17+R16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:R16),0)</f>
         <v/>
       </c>
       <c r="S17" s="13">
-        <f>R17+S16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:S16),0)</f>
         <v/>
       </c>
       <c r="T17" s="13">
-        <f>S17+T16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:T16),0)</f>
         <v/>
       </c>
       <c r="U17" s="13">
-        <f>T17+U16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:U16),0)</f>
         <v/>
       </c>
       <c r="V17" s="13">
-        <f>U17+V16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:V16),0)</f>
         <v/>
       </c>
       <c r="W17" s="13">
-        <f>V17+W16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:W16),0)</f>
         <v/>
       </c>
       <c r="X17" s="13">
-        <f>W17+X16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:X16),0)</f>
         <v/>
       </c>
       <c r="Y17" s="13">
-        <f>X17+Y16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:Y16),0)</f>
         <v/>
       </c>
       <c r="Z17" s="13">
-        <f>Y17+Z16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:Z16),0)</f>
         <v/>
       </c>
       <c r="AA17" s="13">
-        <f>Z17+AA16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AA16),0)</f>
         <v/>
       </c>
       <c r="AB17" s="13">
-        <f>AA17+AB16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AB16),0)</f>
         <v/>
       </c>
       <c r="AC17" s="13">
-        <f>AB17+AC16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AC16),0)</f>
         <v/>
       </c>
       <c r="AD17" s="13">
-        <f>AC17+AD16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AD16),0)</f>
         <v/>
       </c>
       <c r="AE17" s="13">
-        <f>AD17+AE16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AE16),0)</f>
         <v/>
       </c>
       <c r="AF17" s="13">
-        <f>AE17+AF16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AF16),0)</f>
         <v/>
       </c>
       <c r="AG17" s="13">
-        <f>AF17+AG16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AG16),0)</f>
         <v/>
       </c>
       <c r="AH17" s="13">
-        <f>AG17+AH16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AH16),0)</f>
         <v/>
       </c>
       <c r="AI17" s="13">
-        <f>AH17+AI16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AI16),0)</f>
         <v/>
       </c>
       <c r="AJ17" s="13">
-        <f>AI17+AJ16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AJ16),0)</f>
         <v/>
       </c>
       <c r="AK17" s="13">
-        <f>AJ17+AK16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AK16),0)</f>
         <v/>
       </c>
       <c r="AL17" s="13">
-        <f>AK17+AL16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AL16),0)</f>
         <v/>
       </c>
       <c r="AM17" s="13">
-        <f>AL17+AM16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AM16),0)</f>
         <v/>
       </c>
       <c r="AN17" s="13">
-        <f>AM17+AN16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AN16),0)</f>
         <v/>
       </c>
       <c r="AO17" s="13">
-        <f>AN17+AO16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AO16),0)</f>
         <v/>
       </c>
       <c r="AP17" s="13">
-        <f>AO17+AP16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AP16),0)</f>
         <v/>
       </c>
       <c r="AQ17" s="13">
-        <f>AP17+AQ16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AQ16),0)</f>
         <v/>
       </c>
       <c r="AR17" s="13">
-        <f>AQ17+AR16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AR16),0)</f>
         <v/>
       </c>
       <c r="AS17" s="13">
-        <f>AR17+AS16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AS16),0)</f>
         <v/>
       </c>
       <c r="AT17" s="13">
-        <f>AS17+AT16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AT16),0)</f>
         <v/>
       </c>
       <c r="AU17" s="13">
-        <f>AT17+AU16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AU16),0)</f>
         <v/>
       </c>
       <c r="AV17" s="13">
-        <f>AU17+AV16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AV16),0)</f>
         <v/>
       </c>
       <c r="AW17" s="13">
-        <f>AV17+AW16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AW16),0)</f>
         <v/>
       </c>
       <c r="AX17" s="13">
-        <f>AW17+AX16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AX16),0)</f>
         <v/>
       </c>
       <c r="AY17" s="13">
-        <f>AX17+AY16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AY16),0)</f>
         <v/>
       </c>
       <c r="AZ17" s="13">
-        <f>AY17+AZ16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:AZ16),0)</f>
         <v/>
       </c>
       <c r="BA17" s="13">
-        <f>AZ17+BA16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BA16),0)</f>
         <v/>
       </c>
       <c r="BB17" s="13">
-        <f>BA17+BB16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BB16),0)</f>
         <v/>
       </c>
       <c r="BC17" s="13">
-        <f>BB17+BC16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BC16),0)</f>
         <v/>
       </c>
       <c r="BD17" s="13">
-        <f>BC17+BD16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BD16),0)</f>
         <v/>
       </c>
       <c r="BE17" s="13">
-        <f>BD17+BE16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BE16),0)</f>
         <v/>
       </c>
       <c r="BF17" s="13">
-        <f>BE17+BF16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BF16),0)</f>
         <v/>
       </c>
       <c r="BG17" s="13">
-        <f>BF17+BG16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BG16),0)</f>
         <v/>
       </c>
       <c r="BH17" s="13">
-        <f>BG17+BH16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BH16),0)</f>
         <v/>
       </c>
       <c r="BI17" s="13">
-        <f>BH17+BI16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BI16),0)</f>
         <v/>
       </c>
       <c r="BJ17" s="13">
-        <f>BI17+BJ16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BJ16),0)</f>
         <v/>
       </c>
       <c r="BK17" s="13">
-        <f>BJ17+BK16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BK16),0)</f>
         <v/>
       </c>
       <c r="BL17" s="13">
-        <f>BK17+BL16</f>
+        <f>ROUNDDOWN(Assumptions!$F$72+SUM($E16:BL16),0)</f>
         <v/>
       </c>
       <c r="BN17" s="68">
@@ -24200,6 +24200,11 @@
         <f>BL17</f>
         <v/>
       </c>
+      <c r="BT17" s="30" t="inlineStr">
+        <is>
+          <t>whole people only, so half a rep a month means one every second month</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="inlineStr">
@@ -24481,277 +24486,277 @@
     <row r="19">
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Installer partners signed</t>
+          <t>Partner signing rate</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>partners</t>
-        </is>
-      </c>
-      <c r="E19" s="13">
+          <t>partners/month</t>
+        </is>
+      </c>
+      <c r="E19" s="66">
         <f>IF(E$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(E$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="F19" s="13">
+      <c r="F19" s="66">
         <f>IF(F$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(F$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="G19" s="13">
+      <c r="G19" s="66">
         <f>IF(G$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(G$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="H19" s="13">
+      <c r="H19" s="66">
         <f>IF(H$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(H$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="I19" s="13">
+      <c r="I19" s="66">
         <f>IF(I$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(I$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="J19" s="13">
+      <c r="J19" s="66">
         <f>IF(J$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(J$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="K19" s="13">
+      <c r="K19" s="66">
         <f>IF(K$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(K$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="L19" s="13">
+      <c r="L19" s="66">
         <f>IF(L$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(L$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="M19" s="13">
+      <c r="M19" s="66">
         <f>IF(M$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(M$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="N19" s="13">
+      <c r="N19" s="66">
         <f>IF(N$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(N$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="O19" s="13">
+      <c r="O19" s="66">
         <f>IF(O$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(O$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="P19" s="13">
+      <c r="P19" s="66">
         <f>IF(P$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(P$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="Q19" s="13">
+      <c r="Q19" s="66">
         <f>IF(Q$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(Q$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="R19" s="13">
+      <c r="R19" s="66">
         <f>IF(R$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(R$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="S19" s="13">
+      <c r="S19" s="66">
         <f>IF(S$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(S$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="T19" s="13">
+      <c r="T19" s="66">
         <f>IF(T$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(T$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="U19" s="13">
+      <c r="U19" s="66">
         <f>IF(U$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(U$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="V19" s="13">
+      <c r="V19" s="66">
         <f>IF(V$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(V$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="W19" s="13">
+      <c r="W19" s="66">
         <f>IF(W$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(W$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="X19" s="13">
+      <c r="X19" s="66">
         <f>IF(X$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(X$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="Y19" s="13">
+      <c r="Y19" s="66">
         <f>IF(Y$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(Y$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="Z19" s="13">
+      <c r="Z19" s="66">
         <f>IF(Z$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(Z$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AA19" s="13">
+      <c r="AA19" s="66">
         <f>IF(AA$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AA$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AB19" s="13">
+      <c r="AB19" s="66">
         <f>IF(AB$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AB$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AC19" s="13">
+      <c r="AC19" s="66">
         <f>IF(AC$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AC$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AD19" s="13">
+      <c r="AD19" s="66">
         <f>IF(AD$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AD$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AE19" s="13">
+      <c r="AE19" s="66">
         <f>IF(AE$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AE$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AF19" s="13">
+      <c r="AF19" s="66">
         <f>IF(AF$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AF$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AG19" s="13">
+      <c r="AG19" s="66">
         <f>IF(AG$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AG$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AH19" s="13">
+      <c r="AH19" s="66">
         <f>IF(AH$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AH$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AI19" s="13">
+      <c r="AI19" s="66">
         <f>IF(AI$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AI$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AJ19" s="13">
+      <c r="AJ19" s="66">
         <f>IF(AJ$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AJ$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AK19" s="13">
+      <c r="AK19" s="66">
         <f>IF(AK$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AK$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AL19" s="13">
+      <c r="AL19" s="66">
         <f>IF(AL$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AL$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AM19" s="13">
+      <c r="AM19" s="66">
         <f>IF(AM$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AM$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AN19" s="13">
+      <c r="AN19" s="66">
         <f>IF(AN$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AN$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AO19" s="13">
+      <c r="AO19" s="66">
         <f>IF(AO$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AO$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AP19" s="13">
+      <c r="AP19" s="66">
         <f>IF(AP$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AP$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AQ19" s="13">
+      <c r="AQ19" s="66">
         <f>IF(AQ$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AQ$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AR19" s="13">
+      <c r="AR19" s="66">
         <f>IF(AR$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AR$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AS19" s="13">
+      <c r="AS19" s="66">
         <f>IF(AS$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AS$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AT19" s="13">
+      <c r="AT19" s="66">
         <f>IF(AT$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AT$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AU19" s="13">
+      <c r="AU19" s="66">
         <f>IF(AU$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AU$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AV19" s="13">
+      <c r="AV19" s="66">
         <f>IF(AV$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AV$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AW19" s="13">
+      <c r="AW19" s="66">
         <f>IF(AW$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AW$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AX19" s="13">
+      <c r="AX19" s="66">
         <f>IF(AX$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AX$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AY19" s="13">
+      <c r="AY19" s="66">
         <f>IF(AY$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AY$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="AZ19" s="13">
+      <c r="AZ19" s="66">
         <f>IF(AZ$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(AZ$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BA19" s="13">
+      <c r="BA19" s="66">
         <f>IF(BA$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BA$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BB19" s="13">
+      <c r="BB19" s="66">
         <f>IF(BB$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BB$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BC19" s="13">
+      <c r="BC19" s="66">
         <f>IF(BC$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BC$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BD19" s="13">
+      <c r="BD19" s="66">
         <f>IF(BD$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BD$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BE19" s="13">
+      <c r="BE19" s="66">
         <f>IF(BE$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BE$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BF19" s="13">
+      <c r="BF19" s="66">
         <f>IF(BF$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BF$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BG19" s="13">
+      <c r="BG19" s="66">
         <f>IF(BG$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BG$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BH19" s="13">
+      <c r="BH19" s="66">
         <f>IF(BH$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BH$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BI19" s="13">
+      <c r="BI19" s="66">
         <f>IF(BI$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BI$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BJ19" s="13">
+      <c r="BJ19" s="66">
         <f>IF(BJ$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BJ$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BK19" s="13">
+      <c r="BK19" s="66">
         <f>IF(BK$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BK$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BL19" s="13">
+      <c r="BL19" s="66">
         <f>IF(BL$3&lt;Assumptions!$F$13,0,HLOOKUP(YEAR(BL$3),Assumptions!$D$63:$H$66,4,FALSE))</f>
         <v/>
       </c>
-      <c r="BN19" s="68">
+      <c r="BN19" s="67">
         <f>SUM(E19:P19)</f>
         <v/>
       </c>
-      <c r="BO19" s="68">
+      <c r="BO19" s="67">
         <f>SUM(Q19:AB19)</f>
         <v/>
       </c>
-      <c r="BP19" s="68">
+      <c r="BP19" s="67">
         <f>SUM(AC19:AN19)</f>
         <v/>
       </c>
-      <c r="BQ19" s="68">
+      <c r="BQ19" s="67">
         <f>SUM(AO19:AZ19)</f>
         <v/>
       </c>
-      <c r="BR19" s="68">
+      <c r="BR19" s="67">
         <f>SUM(BA19:BL19)</f>
         <v/>
       </c>
       <c r="BT19" s="30" t="inlineStr">
         <is>
-          <t>no partner intros before the first month we can sell</t>
+          <t>the planned rate, which can be less than one a month</t>
         </is>
       </c>
     </row>
@@ -24767,243 +24772,243 @@
         </is>
       </c>
       <c r="E20" s="13">
-        <f>Assumptions!$F$74+E19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:E19),0)</f>
         <v/>
       </c>
       <c r="F20" s="13">
-        <f>E20+F19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:F19),0)</f>
         <v/>
       </c>
       <c r="G20" s="13">
-        <f>F20+G19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:G19),0)</f>
         <v/>
       </c>
       <c r="H20" s="13">
-        <f>G20+H19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:H19),0)</f>
         <v/>
       </c>
       <c r="I20" s="13">
-        <f>H20+I19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:I19),0)</f>
         <v/>
       </c>
       <c r="J20" s="13">
-        <f>I20+J19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:J19),0)</f>
         <v/>
       </c>
       <c r="K20" s="13">
-        <f>J20+K19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:K19),0)</f>
         <v/>
       </c>
       <c r="L20" s="13">
-        <f>K20+L19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:L19),0)</f>
         <v/>
       </c>
       <c r="M20" s="13">
-        <f>L20+M19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:M19),0)</f>
         <v/>
       </c>
       <c r="N20" s="13">
-        <f>M20+N19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:N19),0)</f>
         <v/>
       </c>
       <c r="O20" s="13">
-        <f>N20+O19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:O19),0)</f>
         <v/>
       </c>
       <c r="P20" s="13">
-        <f>O20+P19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:P19),0)</f>
         <v/>
       </c>
       <c r="Q20" s="13">
-        <f>P20+Q19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:Q19),0)</f>
         <v/>
       </c>
       <c r="R20" s="13">
-        <f>Q20+R19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:R19),0)</f>
         <v/>
       </c>
       <c r="S20" s="13">
-        <f>R20+S19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:S19),0)</f>
         <v/>
       </c>
       <c r="T20" s="13">
-        <f>S20+T19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:T19),0)</f>
         <v/>
       </c>
       <c r="U20" s="13">
-        <f>T20+U19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:U19),0)</f>
         <v/>
       </c>
       <c r="V20" s="13">
-        <f>U20+V19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:V19),0)</f>
         <v/>
       </c>
       <c r="W20" s="13">
-        <f>V20+W19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:W19),0)</f>
         <v/>
       </c>
       <c r="X20" s="13">
-        <f>W20+X19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:X19),0)</f>
         <v/>
       </c>
       <c r="Y20" s="13">
-        <f>X20+Y19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:Y19),0)</f>
         <v/>
       </c>
       <c r="Z20" s="13">
-        <f>Y20+Z19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:Z19),0)</f>
         <v/>
       </c>
       <c r="AA20" s="13">
-        <f>Z20+AA19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AA19),0)</f>
         <v/>
       </c>
       <c r="AB20" s="13">
-        <f>AA20+AB19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AB19),0)</f>
         <v/>
       </c>
       <c r="AC20" s="13">
-        <f>AB20+AC19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AC19),0)</f>
         <v/>
       </c>
       <c r="AD20" s="13">
-        <f>AC20+AD19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AD19),0)</f>
         <v/>
       </c>
       <c r="AE20" s="13">
-        <f>AD20+AE19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AE19),0)</f>
         <v/>
       </c>
       <c r="AF20" s="13">
-        <f>AE20+AF19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AF19),0)</f>
         <v/>
       </c>
       <c r="AG20" s="13">
-        <f>AF20+AG19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AG19),0)</f>
         <v/>
       </c>
       <c r="AH20" s="13">
-        <f>AG20+AH19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AH19),0)</f>
         <v/>
       </c>
       <c r="AI20" s="13">
-        <f>AH20+AI19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AI19),0)</f>
         <v/>
       </c>
       <c r="AJ20" s="13">
-        <f>AI20+AJ19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AJ19),0)</f>
         <v/>
       </c>
       <c r="AK20" s="13">
-        <f>AJ20+AK19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AK19),0)</f>
         <v/>
       </c>
       <c r="AL20" s="13">
-        <f>AK20+AL19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AL19),0)</f>
         <v/>
       </c>
       <c r="AM20" s="13">
-        <f>AL20+AM19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AM19),0)</f>
         <v/>
       </c>
       <c r="AN20" s="13">
-        <f>AM20+AN19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AN19),0)</f>
         <v/>
       </c>
       <c r="AO20" s="13">
-        <f>AN20+AO19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AO19),0)</f>
         <v/>
       </c>
       <c r="AP20" s="13">
-        <f>AO20+AP19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AP19),0)</f>
         <v/>
       </c>
       <c r="AQ20" s="13">
-        <f>AP20+AQ19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AQ19),0)</f>
         <v/>
       </c>
       <c r="AR20" s="13">
-        <f>AQ20+AR19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AR19),0)</f>
         <v/>
       </c>
       <c r="AS20" s="13">
-        <f>AR20+AS19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AS19),0)</f>
         <v/>
       </c>
       <c r="AT20" s="13">
-        <f>AS20+AT19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AT19),0)</f>
         <v/>
       </c>
       <c r="AU20" s="13">
-        <f>AT20+AU19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AU19),0)</f>
         <v/>
       </c>
       <c r="AV20" s="13">
-        <f>AU20+AV19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AV19),0)</f>
         <v/>
       </c>
       <c r="AW20" s="13">
-        <f>AV20+AW19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AW19),0)</f>
         <v/>
       </c>
       <c r="AX20" s="13">
-        <f>AW20+AX19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AX19),0)</f>
         <v/>
       </c>
       <c r="AY20" s="13">
-        <f>AX20+AY19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AY19),0)</f>
         <v/>
       </c>
       <c r="AZ20" s="13">
-        <f>AY20+AZ19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:AZ19),0)</f>
         <v/>
       </c>
       <c r="BA20" s="13">
-        <f>AZ20+BA19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BA19),0)</f>
         <v/>
       </c>
       <c r="BB20" s="13">
-        <f>BA20+BB19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BB19),0)</f>
         <v/>
       </c>
       <c r="BC20" s="13">
-        <f>BB20+BC19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BC19),0)</f>
         <v/>
       </c>
       <c r="BD20" s="13">
-        <f>BC20+BD19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BD19),0)</f>
         <v/>
       </c>
       <c r="BE20" s="13">
-        <f>BD20+BE19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BE19),0)</f>
         <v/>
       </c>
       <c r="BF20" s="13">
-        <f>BE20+BF19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BF19),0)</f>
         <v/>
       </c>
       <c r="BG20" s="13">
-        <f>BF20+BG19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BG19),0)</f>
         <v/>
       </c>
       <c r="BH20" s="13">
-        <f>BG20+BH19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BH19),0)</f>
         <v/>
       </c>
       <c r="BI20" s="13">
-        <f>BH20+BI19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BI19),0)</f>
         <v/>
       </c>
       <c r="BJ20" s="13">
-        <f>BI20+BJ19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BJ19),0)</f>
         <v/>
       </c>
       <c r="BK20" s="13">
-        <f>BJ20+BK19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BK19),0)</f>
         <v/>
       </c>
       <c r="BL20" s="13">
-        <f>BK20+BL19</f>
+        <f>ROUNDDOWN(Assumptions!$F$74+SUM($E19:BL19),0)</f>
         <v/>
       </c>
       <c r="BN20" s="68">
@@ -25025,6 +25030,11 @@
       <c r="BR20" s="68">
         <f>BL20</f>
         <v/>
+      </c>
+      <c r="BT20" s="30" t="inlineStr">
+        <is>
+          <t>whole partners only, signed as the running total passes each whole number</t>
+        </is>
       </c>
     </row>
     <row r="21">

</xml_diff>